<commit_message>
Update generated Excel file
</commit_message>
<xml_diff>
--- a/dbc_signals.xlsx
+++ b/dbc_signals.xlsx
@@ -439,10 +439,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -458,7 +458,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Message: Front</t>
+          <t>Message: Pedal_Box</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -468,7 +468,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Sender(s): Aquisition_board1</t>
+          <t>Sender(s): Aquisition_Board1</t>
         </is>
       </c>
     </row>
@@ -532,14 +532,14 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>APPS</t>
+          <t>APPS1</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
@@ -550,20 +550,16 @@
         <v>0</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="3" t="n">
-        <v>100</v>
-      </c>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>bits</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr"/>
@@ -571,14 +567,14 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>hydraulic_brake_pressure</t>
+          <t>APPS2</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
@@ -589,7 +585,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>0</v>
@@ -598,125 +594,129 @@
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>bar</t>
+          <t>bits</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr"/>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>bots</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Intel</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6"/>
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Message: Front_Wheel_L</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>ID: 0x720</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>Sender(s): Aquisition_Board2</t>
+        </is>
+      </c>
+    </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>Message: F_left</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>ID: 0x720</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="inlineStr">
-        <is>
-          <t>Sender(s): Aquisition_board2</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Signal Name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Start Bit</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Length (bits)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Byte Order</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Signed</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Offset</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Choices</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Signal Name</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Start Bit</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Length (bits)</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Byte Order</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Signed</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Factor</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Offset</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Min</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Choices</t>
-        </is>
-      </c>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>wheel_speed</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Km/h</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>wheel_speed</t>
+          <t>tire_temp</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>8</v>
@@ -739,7 +739,7 @@
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Km/h</t>
+          <t>º</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr"/>
@@ -747,11 +747,11 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>tire_temp</t>
+          <t>Brake_disc_temp</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>8</v>
@@ -782,11 +782,11 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Brake_disc_temp</t>
+          <t>wheel_angle</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>8</v>
@@ -814,124 +814,120 @@
       </c>
       <c r="K11" s="3" t="inlineStr"/>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>wheel_angle</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="C12" s="3" t="n">
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Message: Front_Wheel_R</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>ID: 0x730</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>Sender(s): Aquisition_Board3</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Signal Name</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Start Bit</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Length (bits)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Byte Order</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Signed</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Offset</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Choices</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>wheel_speed</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Intel</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="F12" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="n"/>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>º</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>Message: F_right</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
-        <is>
-          <t>ID: 0x730</t>
-        </is>
-      </c>
-      <c r="C14" s="1" t="inlineStr">
-        <is>
-          <t>Sender(s): Aquisition_board3</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Signal Name</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Start Bit</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Length (bits)</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Byte Order</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Signed</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Factor</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Offset</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Min</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Choices</t>
-        </is>
-      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="n"/>
+      <c r="K15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>wheel_speed</t>
+          <t>tire_temp</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>8</v>
@@ -958,11 +954,11 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>tire_temp</t>
+          <t>Brake_disc_temp</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>8</v>
@@ -989,11 +985,11 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Brake_disc_temp</t>
+          <t>wheel_angle</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>8</v>
@@ -1017,120 +1013,120 @@
       <c r="J18" s="3" t="n"/>
       <c r="K18" s="3" t="inlineStr"/>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>wheel_angle</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>Intel</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="F19" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="n"/>
-      <c r="J19" s="3" t="n"/>
-      <c r="K19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20"/>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>Message: Data_Box</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>ID: 0x740</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>Sender(s): Aquisition_Board4</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>Message: data_box</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
-        <is>
-          <t>ID: 0x740</t>
-        </is>
-      </c>
-      <c r="C21" s="1" t="inlineStr">
-        <is>
-          <t>Sender(s): Aquisition_board4</t>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Signal Name</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Start Bit</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Length (bits)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Byte Order</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Signed</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Offset</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Choices</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Signal Name</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Start Bit</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Length (bits)</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Byte Order</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Signed</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Factor</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Offset</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>Min</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Choices</t>
-        </is>
-      </c>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>suspension_level_left</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="3" t="n"/>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="n"/>
+      <c r="K22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>suspension_level_left</t>
+          <t>suspension_level_right</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="C23" s="3" t="n">
         <v>16</v>
@@ -1154,120 +1150,120 @@
       <c r="J23" s="3" t="n"/>
       <c r="K23" s="3" t="inlineStr"/>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>suspension_level_right</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="C24" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Intel</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="F24" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="3" t="n"/>
-      <c r="J24" s="3" t="n"/>
-      <c r="K24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25"/>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>Message: Rear_Wheel_L</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>ID: 0x750</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>Sender(s): Aquisition_Board5</t>
+        </is>
+      </c>
+    </row>
     <row r="26">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>Message: Side_panel</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
-        <is>
-          <t>ID: 0x750</t>
-        </is>
-      </c>
-      <c r="C26" s="1" t="inlineStr">
-        <is>
-          <t>Sender(s): Aquisition_board7</t>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Signal Name</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Start Bit</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Length (bits)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Byte Order</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Signed</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Offset</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Choices</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Signal Name</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Start Bit</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Length (bits)</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Byte Order</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>Signed</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Factor</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>Offset</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>Min</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>Choices</t>
-        </is>
-      </c>
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Shutdown_circuit</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="3" t="n"/>
+      <c r="I27" s="3" t="n"/>
+      <c r="J27" s="3" t="n"/>
+      <c r="K27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Shutdown_circuit</t>
+          <t>mission_select</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C28" s="3" t="n">
         <v>1</v>
@@ -1294,11 +1290,11 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>mission_select</t>
+          <t>ignition</t>
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C29" s="3" t="n">
         <v>1</v>
@@ -1322,123 +1318,127 @@
       <c r="J29" s="3" t="n"/>
       <c r="K29" s="3" t="inlineStr"/>
     </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>ignition</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C30" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>Intel</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="F30" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G30" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="3" t="n"/>
-      <c r="I30" s="3" t="n"/>
-      <c r="J30" s="3" t="n"/>
-      <c r="K30" s="3" t="inlineStr"/>
-    </row>
-    <row r="31"/>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>Message: Rear_Wheel_R</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>ID: 0x760</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>Sender(s): Aquisition_Board6</t>
+        </is>
+      </c>
+    </row>
     <row r="32">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>Message: Rear_pressure</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="inlineStr">
-        <is>
-          <t>ID: 0x760</t>
-        </is>
-      </c>
-      <c r="C32" s="1" t="inlineStr">
-        <is>
-          <t>Sender(s): Aquisition_board8</t>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Signal Name</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Start Bit</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Length (bits)</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Byte Order</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Signed</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Offset</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Choices</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Signal Name</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Start Bit</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Length (bits)</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Byte Order</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Signed</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>Factor</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>Offset</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>Min</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>Choices</t>
-        </is>
-      </c>
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Hydrauli_brake_pressure</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="3" t="n"/>
+      <c r="I33" s="3" t="n"/>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Hydrauli_brake_pressure</t>
+          <t>NTC1</t>
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
@@ -1458,7 +1458,7 @@
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>bar</t>
+          <t>º</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr"/>
@@ -1466,11 +1466,11 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>NTC1</t>
+          <t>NTC2</t>
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C35" s="3" t="n">
         <v>8</v>
@@ -1501,11 +1501,11 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>NTC2</t>
+          <t>NTC3</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C36" s="3" t="n">
         <v>8</v>
@@ -1536,11 +1536,11 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>NTC3</t>
+          <t>NTC4</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="C37" s="3" t="n">
         <v>8</v>
@@ -1571,11 +1571,11 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>NTC4</t>
+          <t>NTC5</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="C38" s="3" t="n">
         <v>8</v>
@@ -1606,11 +1606,11 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>NTC5</t>
+          <t>NTC6</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="C39" s="3" t="n">
         <v>8</v>
@@ -1638,127 +1638,123 @@
       </c>
       <c r="K39" s="3" t="inlineStr"/>
     </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>NTC6</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="n">
-        <v>56</v>
-      </c>
-      <c r="C40" s="3" t="n">
+    <row r="40"/>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>Message: Central_Rear</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>ID: 0x8</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>Sender(s): Aquisition_Board7</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Signal Name</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Start Bit</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Length (bits)</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Byte Order</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Signed</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Offset</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Choices</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>wheel_speed</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>Intel</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="F40" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G40" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" s="3" t="n"/>
-      <c r="I40" s="3" t="n"/>
-      <c r="J40" s="3" t="inlineStr">
-        <is>
-          <t>º</t>
-        </is>
-      </c>
-      <c r="K40" s="3" t="inlineStr"/>
-    </row>
-    <row r="41"/>
-    <row r="42">
-      <c r="A42" s="1" t="inlineStr">
-        <is>
-          <t>Message: Rear_left</t>
-        </is>
-      </c>
-      <c r="B42" s="1" t="inlineStr">
-        <is>
-          <t>ID: 0x8</t>
-        </is>
-      </c>
-      <c r="C42" s="1" t="inlineStr">
-        <is>
-          <t>Sender(s): Aquisition_board6</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Signal Name</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Start Bit</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Length (bits)</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Byte Order</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>Signed</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>Factor</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>Offset</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>Min</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
-      <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="K43" s="2" t="inlineStr">
-        <is>
-          <t>Choices</t>
-        </is>
-      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="3" t="n"/>
+      <c r="I43" s="3" t="n"/>
+      <c r="J43" s="3" t="n"/>
+      <c r="K43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>wheel_speed</t>
+          <t>Tire_temp</t>
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C44" s="3" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
@@ -1769,7 +1765,7 @@
         <v>0</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G44" s="3" t="n">
         <v>0</v>
@@ -1782,11 +1778,11 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Tire_temp</t>
+          <t>Brake_disk_temp</t>
         </is>
       </c>
       <c r="B45" s="3" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="C45" s="3" t="n">
         <v>16</v>
@@ -1809,37 +1805,6 @@
       <c r="I45" s="3" t="n"/>
       <c r="J45" s="3" t="n"/>
       <c r="K45" s="3" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>Brake_disk_temp</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="C46" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>Intel</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="F46" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="G46" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="3" t="n"/>
-      <c r="I46" s="3" t="n"/>
-      <c r="J46" s="3" t="n"/>
-      <c r="K46" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1852,12 +1817,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
@@ -2610,6 +2575,680 @@
       </c>
       <c r="K22" s="3" t="inlineStr"/>
     </row>
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Message: AQT1</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>ID: 0x710</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>Sender(s): Aquisition_Board1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Signal Name</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Start Bit</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Length (bits)</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Byte Order</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Signed</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Offset</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Choices</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>BRK_PRESS</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="n"/>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>RES</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="3" t="n"/>
+      <c r="I27" s="3" t="n"/>
+      <c r="J27" s="3" t="n"/>
+      <c r="K27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>BOTS</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="3" t="n"/>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+      <c r="K28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Message: AQT2</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>ID: 0x720</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>Sender(s): Aquisition_Board2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Signal Name</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Start Bit</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Length (bits)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Byte Order</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Signed</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Offset</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Choices</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>WHEEL_ANGLE</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="3" t="n"/>
+      <c r="I32" s="3" t="n"/>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>º</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33"/>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>Message: AQT3</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="inlineStr">
+        <is>
+          <t>ID: 0x730</t>
+        </is>
+      </c>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>Sender(s): Aquisition_Board3</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Signal Name</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Start Bit</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Length (bits)</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Byte Order</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Signed</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Offset</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Choices</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>WHEEL_ANGLE</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="3" t="n"/>
+      <c r="I36" s="3" t="n"/>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>º</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>Message: AQT4</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>ID: 0x740</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>Sender(s): Aquisition_Board4</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Signal Name</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Start Bit</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Length (bits)</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Byte Order</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Signed</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Offset</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Choices</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>ST_ANGLE</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="3" t="n"/>
+      <c r="I40" s="3" t="n"/>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>º</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>INERTIA</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="3" t="n"/>
+      <c r="I41" s="3" t="n"/>
+      <c r="J41" s="3" t="n"/>
+      <c r="K41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>EMER_BUTTON</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="3" t="n"/>
+      <c r="I42" s="3" t="n"/>
+      <c r="J42" s="3" t="n"/>
+      <c r="K42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43"/>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>Message: AQT7</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>ID: 0x770</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>Sender(s): Aquisition_Board7</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Signal Name</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Start Bit</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Length (bits)</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Byte Order</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Signed</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Offset</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>Choices</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>BRK_PRESS</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="3" t="n"/>
+      <c r="I46" s="3" t="n"/>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2621,12 +3260,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1042"/>
+  <dimension ref="A1:K1052"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
@@ -35013,6 +35652,288 @@
       </c>
       <c r="K1042" s="3" t="inlineStr"/>
     </row>
+    <row r="1043"/>
+    <row r="1044">
+      <c r="A1044" s="1" t="inlineStr">
+        <is>
+          <t>Message: APPS_ADC_Raw</t>
+        </is>
+      </c>
+      <c r="B1044" s="1" t="inlineStr">
+        <is>
+          <t>ID: 0x710</t>
+        </is>
+      </c>
+      <c r="C1044" s="1" t="inlineStr">
+        <is>
+          <t>Sender(s): Aquisition_Board1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" s="2" t="inlineStr">
+        <is>
+          <t>Signal Name</t>
+        </is>
+      </c>
+      <c r="B1045" s="2" t="inlineStr">
+        <is>
+          <t>Start Bit</t>
+        </is>
+      </c>
+      <c r="C1045" s="2" t="inlineStr">
+        <is>
+          <t>Length (bits)</t>
+        </is>
+      </c>
+      <c r="D1045" s="2" t="inlineStr">
+        <is>
+          <t>Byte Order</t>
+        </is>
+      </c>
+      <c r="E1045" s="2" t="inlineStr">
+        <is>
+          <t>Signed</t>
+        </is>
+      </c>
+      <c r="F1045" s="2" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="G1045" s="2" t="inlineStr">
+        <is>
+          <t>Offset</t>
+        </is>
+      </c>
+      <c r="H1045" s="2" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="I1045" s="2" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="J1045" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K1045" s="2" t="inlineStr">
+        <is>
+          <t>Choices</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" s="3" t="inlineStr">
+        <is>
+          <t>APPS1</t>
+        </is>
+      </c>
+      <c r="B1046" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1046" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D1046" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E1046" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F1046" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G1046" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1046" s="3" t="n"/>
+      <c r="I1046" s="3" t="n"/>
+      <c r="J1046" s="3" t="inlineStr">
+        <is>
+          <t>bits</t>
+        </is>
+      </c>
+      <c r="K1046" s="3" t="inlineStr"/>
+    </row>
+    <row r="1047">
+      <c r="A1047" s="3" t="inlineStr">
+        <is>
+          <t>APPS2</t>
+        </is>
+      </c>
+      <c r="B1047" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="C1047" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D1047" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E1047" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F1047" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G1047" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1047" s="3" t="n"/>
+      <c r="I1047" s="3" t="n"/>
+      <c r="J1047" s="3" t="inlineStr">
+        <is>
+          <t>bits</t>
+        </is>
+      </c>
+      <c r="K1047" s="3" t="inlineStr"/>
+    </row>
+    <row r="1048"/>
+    <row r="1049">
+      <c r="A1049" s="1" t="inlineStr">
+        <is>
+          <t>Message: DashBoard</t>
+        </is>
+      </c>
+      <c r="B1049" s="1" t="inlineStr">
+        <is>
+          <t>ID: 0x740</t>
+        </is>
+      </c>
+      <c r="C1049" s="1" t="inlineStr">
+        <is>
+          <t>Sender(s): Aquisition_Board4</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" s="2" t="inlineStr">
+        <is>
+          <t>Signal Name</t>
+        </is>
+      </c>
+      <c r="B1050" s="2" t="inlineStr">
+        <is>
+          <t>Start Bit</t>
+        </is>
+      </c>
+      <c r="C1050" s="2" t="inlineStr">
+        <is>
+          <t>Length (bits)</t>
+        </is>
+      </c>
+      <c r="D1050" s="2" t="inlineStr">
+        <is>
+          <t>Byte Order</t>
+        </is>
+      </c>
+      <c r="E1050" s="2" t="inlineStr">
+        <is>
+          <t>Signed</t>
+        </is>
+      </c>
+      <c r="F1050" s="2" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="G1050" s="2" t="inlineStr">
+        <is>
+          <t>Offset</t>
+        </is>
+      </c>
+      <c r="H1050" s="2" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="I1050" s="2" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="J1050" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K1050" s="2" t="inlineStr">
+        <is>
+          <t>Choices</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" s="3" t="inlineStr">
+        <is>
+          <t>Ignition</t>
+        </is>
+      </c>
+      <c r="B1051" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1051" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1051" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E1051" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F1051" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1051" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1051" s="3" t="n"/>
+      <c r="I1051" s="3" t="n"/>
+      <c r="J1051" s="3" t="n"/>
+      <c r="K1051" s="3" t="inlineStr"/>
+    </row>
+    <row r="1052">
+      <c r="A1052" s="3" t="inlineStr">
+        <is>
+          <t>Ready_To_Drive</t>
+        </is>
+      </c>
+      <c r="B1052" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1052" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1052" s="3" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="E1052" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F1052" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1052" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1052" s="3" t="n"/>
+      <c r="I1052" s="3" t="n"/>
+      <c r="J1052" s="3" t="n"/>
+      <c r="K1052" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>